<commit_message>
Add total GitHub platform activity quarterly time series (Q1 2022 – Q1 2026)
New sheet 'GitHub Platform Activity' in the Excel workbook with:

- Global git pushes: Official data from GitHub Innovation Graph
  (github/innovationgraph repo, git_pushes.csv) covering Q1 2020 – Q3 2025.
  Q4 2025 estimated from Octoverse 2025 annual total (~1B commits, +25.1%
  YoY). Q1 2026 estimated at ~28% YoY growth trajectory.

- Active developers: 89.6M (Q1 2022) → 210M+ (Q1 2026 est.); 36M new
  developers joined in 2025 alone (one per second)

- Total repositories: 230M (Q1 2022) → 482M (Q1 2026 est.); 230+ new
  repos created per minute in 2025

- QoQ and YoY growth rates, pushes-per-developer ratio

- Annual summary table (2022: 599M pushes → 2025: 942M pushes)

- Stacked bar chart for quarterly git pushes

Also adds github_platform_activity_quarterly.csv for programmatic access.
Updated README with new data source documentation.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mcp_ecosystem_token_usage_correlation.xlsx
+++ b/data/mcp_ecosystem_token_usage_correlation.xlsx
@@ -19,6 +19,7 @@
     <sheet name="LLM Revenue Run-Rate" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="LLM GitHub Commits" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Token Usage by Provider" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="GitHub Platform Activity" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1497,6 +1498,108 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>GitHub Global Git Pushes (Quarterly)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'GitHub Platform Activity'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="333333"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'GitHub Platform Activity'!$A$2:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'GitHub Platform Activity'!$B$2:$B$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Git Pushes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="#,##0,,&quot;M&quot;" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1629,6 +1732,33 @@
       <col>0</col>
       <colOff>0</colOff>
       <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11520000" cy="6480000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="11520000" cy="6480000"/>
@@ -4938,6 +5068,759 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00333333"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Git Pushes
+(Global)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Push QoQ
+Growth</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Push YoY
+Growth</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Active
+Developers</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Dev QoQ
+Growth</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Total
+Repositories</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Pushes per
+Developer</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2022-Q1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>140572256</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.09067307080704778</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.1590825157777029</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>89612163</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.07120588237895831</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>229733614</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2022-Q2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>149717365</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.06505628678250708</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.1738912074275534</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>95043584</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.06061031023210539</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>243339989</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2022-Q3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>146835949</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>-0.01924570339586196</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.2642123768015416</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>100334892</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.05567243760504659</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>256393118</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2022-Q4</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>161464841</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.09962745567163522</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.252774615503373</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>105809362</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.05456197630630832</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>269935545</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2023-Q1</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>172765182</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.06998638793444822</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.2290133694660204</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>112142497</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.05985420269333064</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>283851980</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2023-Q2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>175270480</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.01450117420071373</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.1706756928296194</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>118863203</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.05993005488365388</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>298254607</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2023-Q3</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>165466632</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>-0.05593553460913669</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.1268809384001734</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>125462005</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.0555159362481592</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>311778148</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2023-Q4</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>178868690</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.08099553268238391</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.1077872364795505</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>131883095</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0.05117955830532117</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>326068851</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2024-Q1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>184167232</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.02962252365128859</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.06599738366264107</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>139575994</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.05833119855126245</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>340737253</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2024-Q2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>189331668</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.02804210034497334</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.08022564895126671</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>145646544</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0.04349279432679509</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>355510606</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2024-Q3</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>179232651</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>-0.05334034769080465</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.08319513628584652</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>151993922</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.04358069766488937</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>369639247</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2024-Q4</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>200262211</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.1173310771372789</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.1196046161013422</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>159142080</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0.04702923581378471</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>385466517</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>213071277</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.06396147299102783</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.1569445589538969</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>167884897</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.05493717940597476</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>402290482</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>247828515</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0.1631249340097587</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.3089649376563883</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>177219553</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0.05560152322695244</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>420993825</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2025-Q3</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>250894326</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.01237069511553179</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.3998248901646833</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>189778233</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.07086509240884942</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>440152951</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2025-Q4</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>230201078</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>-0.08247794332343727</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.1494983344611132</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>198000000</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0.04332302430068458</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>460000000</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Estimated from Octoverse 2025 (~1B commits, +25.1% YoY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>272731234</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.1847522017251371</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.2799999973717715</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>210000000</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.06060606060606055</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>482000000</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Estimated (~28% YoY growth trajectory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Annual Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Total Pushes</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>YoY Growth</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Active Devs (YE)</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>598590411</v>
+      </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="3" t="n">
+        <v>105809362</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Innovation Graph</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>692370984</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.1566690198784357</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>131883095</v>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Innovation Graph</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>752993762</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>0.08755823019873987</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>159142080</v>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Innovation Graph</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>941995196</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.2509999996520555</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>198000000</v>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Octoverse 2025: ~1B commits, +25.1% YoY</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A21:E21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9392,7 +10275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -9861,6 +10744,33 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Platform Activity</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Innovation Graph + Octoverse</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>github/innovationgraph CSV data (git_pushes, developers, repos)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Q1 2020 – Q3 2025 official; Q4 2025, Q1 2026 estimated</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Git pushes ≈ commits proxy; Q4 2025 derived from Octoverse annual total</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>